<commit_message>
📊 Weekly RSI Screener Report – 2026-05-23
</commit_message>
<xml_diff>
--- a/docs/Micro250_stocks.xlsx
+++ b/docs/Micro250_stocks.xlsx
@@ -567,7 +567,7 @@
         <v>183.44</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>6428792</v>
+        <v>6428806</v>
       </c>
       <c r="K2" s="4" t="n">
         <v>21536</v>
@@ -606,7 +606,7 @@
         <v>1933.92</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>340211</v>
+        <v>340214</v>
       </c>
       <c r="K3" s="4" t="n">
         <v>17788</v>
@@ -684,7 +684,7 @@
         <v>3540.42</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>1522731</v>
+        <v>1522738</v>
       </c>
       <c r="K5" s="4" t="n">
         <v>24840</v>
@@ -723,7 +723,7 @@
         <v>934.16</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>373720</v>
+        <v>373721</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>10629</v>
@@ -762,7 +762,7 @@
         <v>697.35</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>483591</v>
+        <v>483597</v>
       </c>
       <c r="K7" s="4" t="n">
         <v>8307</v>
@@ -879,7 +879,7 @@
         <v>995.7</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>379596</v>
+        <v>379610</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>11155</v>
@@ -918,7 +918,7 @@
         <v>3859.81</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>151828</v>
+        <v>151829</v>
       </c>
       <c r="K11" s="4" t="n">
         <v>12437</v>
@@ -957,7 +957,7 @@
         <v>2159.04</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>531436</v>
+        <v>531437</v>
       </c>
       <c r="K12" s="4" t="n">
         <v>12397</v>
@@ -996,7 +996,7 @@
         <v>133.61</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>1170635</v>
+        <v>1170638</v>
       </c>
       <c r="K13" s="4" t="n">
         <v>7497</v>
@@ -1035,7 +1035,7 @@
         <v>1213.33</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>338416</v>
+        <v>338425</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>15553</v>
@@ -1074,7 +1074,7 @@
         <v>213</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>3249038</v>
+        <v>3249117</v>
       </c>
       <c r="K15" s="4" t="n">
         <v>10003</v>
@@ -1113,7 +1113,7 @@
         <v>287.34</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>734013</v>
+        <v>734024</v>
       </c>
       <c r="K16" s="4" t="n">
         <v>5985</v>
@@ -1152,7 +1152,7 @@
         <v>1709.9</v>
       </c>
       <c r="J17" s="4" t="n">
-        <v>584364</v>
+        <v>584401</v>
       </c>
       <c r="K17" s="4" t="n">
         <v>13172</v>

</xml_diff>